<commit_message>
Fix Q7. Solution now is defined by correct initial parameters.
</commit_message>
<xml_diff>
--- a/Interim3/ENME473_Q7_BoxDimensions.xlsx
+++ b/Interim3/ENME473_Q7_BoxDimensions.xlsx
@@ -99,13 +99,13 @@
         <v>0</v>
       </c>
       <c r="B2" s="0">
-        <v>749.57490946220378</v>
+        <v>721.18189187126336</v>
       </c>
       <c r="C2" s="0">
-        <v>192.16671859878784</v>
+        <v>317.24983717232072</v>
       </c>
       <c r="D2" s="0">
-        <v>144043.35069533519</v>
+        <v>228794.83776778451</v>
       </c>
     </row>
     <row r="3">
@@ -113,13 +113,13 @@
         <v>5</v>
       </c>
       <c r="B3" s="0">
-        <v>754.35943958072608</v>
+        <v>724.18323456929693</v>
       </c>
       <c r="C3" s="0">
-        <v>271.89271479488105</v>
+        <v>396.5576523318972</v>
       </c>
       <c r="D3" s="0">
-        <v>205104.83595874865</v>
+        <v>287180.40335892001</v>
       </c>
     </row>
     <row r="4">
@@ -127,13 +127,13 @@
         <v>10</v>
       </c>
       <c r="B4" s="0">
-        <v>763.76557912969372</v>
+        <v>733.13865958881252</v>
       </c>
       <c r="C4" s="0">
-        <v>337.07648015038296</v>
+        <v>461.63145515915699</v>
       </c>
       <c r="D4" s="0">
-        <v>257447.41307305594</v>
+        <v>338439.86625941738</v>
       </c>
     </row>
     <row r="5">
@@ -141,13 +141,13 @@
         <v>15</v>
       </c>
       <c r="B5" s="0">
-        <v>776.79992559284892</v>
+        <v>746.13831744707431</v>
       </c>
       <c r="C5" s="0">
-        <v>396.70096919848209</v>
+        <v>521.2474094764558</v>
       </c>
       <c r="D5" s="0">
-        <v>308157.28335599194</v>
+        <v>388922.66508040891</v>
       </c>
     </row>
     <row r="6">
@@ -155,13 +155,13 @@
         <v>20</v>
       </c>
       <c r="B6" s="0">
-        <v>793.12280296662641</v>
+        <v>762.62657541713418</v>
       </c>
       <c r="C6" s="0">
-        <v>452.52553716383</v>
+        <v>577.11257543527108</v>
       </c>
       <c r="D6" s="0">
-        <v>358908.3224493551</v>
+        <v>440121.38703436329</v>
       </c>
     </row>
     <row r="7">
@@ -169,13 +169,13 @@
         <v>25</v>
       </c>
       <c r="B7" s="0">
-        <v>812.51719945469085</v>
+        <v>782.30542345251774</v>
       </c>
       <c r="C7" s="0">
-        <v>504.93607747696467</v>
+        <v>629.59239938160954</v>
       </c>
       <c r="D7" s="0">
-        <v>410269.24757522013</v>
+        <v>492533.54860071675</v>
       </c>
     </row>
     <row r="8">
@@ -183,13 +183,13 @@
         <v>30</v>
       </c>
       <c r="B8" s="0">
-        <v>834.79379463241367</v>
+        <v>804.94920858940031</v>
       </c>
       <c r="C8" s="0">
-        <v>553.88007288036897</v>
+        <v>678.62481498969032</v>
       </c>
       <c r="D8" s="0">
-        <v>462375.64781108103</v>
+        <v>546258.50775507942</v>
       </c>
     </row>
     <row r="9">
@@ -197,13 +197,13 @@
         <v>35</v>
       </c>
       <c r="B9" s="0">
-        <v>859.76312529369409</v>
+        <v>830.351083056721</v>
       </c>
       <c r="C9" s="0">
-        <v>599.13373360342598</v>
+        <v>723.98116758366609</v>
       </c>
       <c r="D9" s="0">
-        <v>515113.09127176105</v>
+        <v>601158.5466157666</v>
       </c>
     </row>
     <row r="10">
@@ -211,13 +211,13 @@
         <v>40</v>
       </c>
       <c r="B10" s="0">
-        <v>887.22578825402184</v>
+        <v>858.30376212375108</v>
       </c>
       <c r="C10" s="0">
-        <v>640.40136484783443</v>
+        <v>765.36322464721445</v>
       </c>
       <c r="D10" s="0">
-        <v>568180.60572607129</v>
+        <v>656914.13510586985</v>
       </c>
     </row>
     <row r="11">
@@ -225,13 +225,13 @@
         <v>45</v>
       </c>
       <c r="B11" s="0">
-        <v>916.96893076443519</v>
+        <v>888.59202279444366</v>
       </c>
       <c r="C11" s="0">
-        <v>677.35870942295401</v>
+        <v>802.44548368011761</v>
       </c>
       <c r="D11" s="0">
-        <v>621116.89152354386</v>
+        <v>713046.65552558145</v>
       </c>
     </row>
     <row r="12">
@@ -239,13 +239,13 @@
         <v>50</v>
       </c>
       <c r="B12" s="0">
-        <v>948.76532462207956</v>
+        <v>920.9899838428878</v>
       </c>
       <c r="C12" s="0">
-        <v>709.67373718544059</v>
+        <v>834.89546231570591</v>
       </c>
       <c r="D12" s="0">
-        <v>673313.83363650891</v>
+        <v>768930.35834864236</v>
       </c>
     </row>
     <row r="13">
@@ -253,13 +253,13 @@
         <v>55</v>
       </c>
       <c r="B13" s="0">
-        <v>982.37362214554162</v>
+        <v>955.26059982514153</v>
       </c>
       <c r="C13" s="0">
-        <v>737.01679849846698</v>
+        <v>862.38359641822478</v>
       </c>
       <c r="D13" s="0">
-        <v>724025.86192304979</v>
+        <v>823801.07159383618</v>
       </c>
     </row>
     <row r="14">
@@ -267,13 +267,13 @@
         <v>60</v>
       </c>
       <c r="B14" s="0">
-        <v>1017.5391703716315</v>
+        <v>991.15628784853254</v>
       </c>
       <c r="C14" s="0">
-        <v>759.0647943571654</v>
+        <v>884.58727644612145</v>
       </c>
       <c r="D14" s="0">
-        <v>772378.16110850312</v>
+        <v>876764.24120038143</v>
       </c>
     </row>
     <row r="15">
@@ -281,13 +281,13 @@
         <v>65</v>
       </c>
       <c r="B15" s="0">
-        <v>1053.9950424142089</v>
+        <v>1028.4201730270577</v>
       </c>
       <c r="C15" s="0">
-        <v>775.50111635450014</v>
+        <v>901.19071837403908</v>
       </c>
       <c r="D15" s="0">
-        <v>817374.33202432771</v>
+        <v>926802.71452060773</v>
       </c>
     </row>
     <row r="16">
@@ -295,13 +295,13 @@
         <v>70</v>
       </c>
       <c r="B16" s="0">
-        <v>1091.4630303772233</v>
+        <v>1066.7876658444998</v>
       </c>
       <c r="C16" s="0">
-        <v>786.01167976574823</v>
+        <v>911.88096269521088</v>
       </c>
       <c r="D16" s="0">
-        <v>857902.6899090152</v>
+        <v>972783.36372165941</v>
       </c>
     </row>
     <row r="17">
@@ -309,13 +309,13 @@
         <v>75</v>
       </c>
       <c r="B17" s="0">
-        <v>1129.6543193869115</v>
+        <v>1105.9881601704744</v>
       </c>
       <c r="C17" s="0">
-        <v>793.79861087035783</v>
+        <v>916.33930775375109</v>
       </c>
       <c r="D17" s="0">
-        <v>896718.02949302993</v>
+        <v>1013460.4250744573</v>
       </c>
     </row>
     <row r="18">
@@ -323,13 +323,13 @@
         <v>80</v>
       </c>
       <c r="B18" s="0">
-        <v>1168.2694286799262</v>
+        <v>1145.7466176480414</v>
       </c>
       <c r="C18" s="0">
-        <v>796.83450709137242</v>
+        <v>914.22639594845941</v>
       </c>
       <c r="D18" s="0">
-        <v>930917.39435208833</v>
+        <v>1047471.8009225064</v>
       </c>
     </row>
     <row r="19">
@@ -337,13 +337,13 @@
         <v>85</v>
       </c>
       <c r="B19" s="0">
-        <v>1206.9966952336056</v>
+        <v>1185.7846637662365</v>
       </c>
       <c r="C19" s="0">
-        <v>793.67001186378479</v>
+        <v>905.15749474800464</v>
       </c>
       <c r="D19" s="0">
-        <v>957957.08142560476</v>
+        <v>1073321.8755652516</v>
       </c>
     </row>
     <row r="20">
@@ -351,13 +351,13 @@
         <v>90</v>
       </c>
       <c r="B20" s="0">
-        <v>1245.5078988954349</v>
+        <v>1225.8204562473786</v>
       </c>
       <c r="C20" s="0">
-        <v>784.04360861304622</v>
+        <v>888.66143150626897</v>
       </c>
       <c r="D20" s="0">
-        <v>976532.50760602986</v>
+        <v>1089339.3614184633</v>
       </c>
     </row>
     <row r="21">
@@ -365,13 +365,13 @@
         <v>95</v>
       </c>
       <c r="B21" s="0">
-        <v>1307.1893226825234</v>
+        <v>1289.3069153111589</v>
       </c>
       <c r="C21" s="0">
-        <v>767.62883396882</v>
+        <v>864.11035824295891</v>
       </c>
       <c r="D21" s="0">
-        <v>1003436.215547277</v>
+        <v>1114103.4604746499</v>
       </c>
     </row>
     <row r="22">
@@ -379,13 +379,13 @@
         <v>100</v>
       </c>
       <c r="B22" s="0">
-        <v>1367.7147950669782</v>
+        <v>1352.0175686629702</v>
       </c>
       <c r="C22" s="0">
-        <v>743.96612021033957</v>
+        <v>830.59353314043449</v>
       </c>
       <c r="D22" s="0">
-        <v>1017533.4696402595</v>
+        <v>1122977.0492237164</v>
       </c>
     </row>
     <row r="23">
@@ -393,13 +393,13 @@
         <v>105</v>
       </c>
       <c r="B23" s="0">
-        <v>1426.3997848583081</v>
+        <v>1413.4252579020172</v>
       </c>
       <c r="C23" s="0">
-        <v>712.33102031441308</v>
+        <v>786.67385182756288</v>
       </c>
       <c r="D23" s="0">
-        <v>1016068.8141243779</v>
+        <v>1111904.6919041462</v>
       </c>
     </row>
     <row r="24">
@@ -407,13 +407,13 @@
         <v>110</v>
       </c>
       <c r="B24" s="0">
-        <v>1482.3338326520243</v>
+        <v>1472.8869020475863</v>
       </c>
       <c r="C24" s="0">
-        <v>671.45323989271492</v>
+        <v>729.86918355829118</v>
       </c>
       <c r="D24" s="0">
-        <v>995317.85453678714</v>
+        <v>1075014.7606711725</v>
       </c>
     </row>
     <row r="25">
@@ -421,13 +421,13 @@
         <v>115</v>
       </c>
       <c r="B25" s="0">
-        <v>1534.0190566554104</v>
+        <v>1529.4108256751295</v>
       </c>
       <c r="C25" s="0">
-        <v>618.82450138813113</v>
+        <v>655.3745328594913</v>
       </c>
       <c r="D25" s="0">
-        <v>949288.57785467559</v>
+        <v>1002336.9054270869</v>
       </c>
     </row>
     <row r="26">
@@ -435,13 +435,13 @@
         <v>120</v>
       </c>
       <c r="B26" s="0">
-        <v>1578.0613435288069</v>
+        <v>1580.75050658341</v>
       </c>
       <c r="C26" s="0">
-        <v>548.54007705640459</v>
+        <v>552.07109398706075</v>
       </c>
       <c r="D26" s="0">
-        <v>865629.89097902505</v>
+        <v>872686.6614901037</v>
       </c>
     </row>
   </sheetData>
@@ -478,13 +478,13 @@
         <v>0</v>
       </c>
       <c r="B2" s="0">
-        <v>749.57490946220378</v>
+        <v>761.23831235875093</v>
       </c>
       <c r="C2" s="0">
-        <v>192.16671859878619</v>
+        <v>227.85929594485208</v>
       </c>
       <c r="D2" s="0">
-        <v>144043.35069533394</v>
+        <v>173455.22590031236</v>
       </c>
     </row>
     <row r="3">
@@ -492,13 +492,13 @@
         <v>5</v>
       </c>
       <c r="B3" s="0">
-        <v>754.35943958072608</v>
+        <v>763.55377057003204</v>
       </c>
       <c r="C3" s="0">
-        <v>271.8927147948815</v>
+        <v>321.59868152706906</v>
       </c>
       <c r="D3" s="0">
-        <v>205104.835958749</v>
+        <v>245557.88589034448</v>
       </c>
     </row>
     <row r="4">
@@ -506,13 +506,13 @@
         <v>10</v>
       </c>
       <c r="B4" s="0">
-        <v>763.76557912969372</v>
+        <v>772.44581823758108</v>
       </c>
       <c r="C4" s="0">
-        <v>337.0764801503833</v>
+        <v>389.13234938420442</v>
       </c>
       <c r="D4" s="0">
-        <v>257447.4130730562</v>
+        <v>300583.65602279408</v>
       </c>
     </row>
     <row r="5">
@@ -520,13 +520,13 @@
         <v>15</v>
       </c>
       <c r="B5" s="0">
-        <v>776.79992559284892</v>
+        <v>785.33569826039775</v>
       </c>
       <c r="C5" s="0">
-        <v>396.70096919848226</v>
+        <v>449.67442900751735</v>
       </c>
       <c r="D5" s="0">
-        <v>308157.28335599206</v>
+        <v>353145.38169446431</v>
       </c>
     </row>
     <row r="6">
@@ -534,13 +534,13 @@
         <v>20</v>
       </c>
       <c r="B6" s="0">
-        <v>793.12280296662641</v>
+        <v>801.66231265908982</v>
       </c>
       <c r="C6" s="0">
-        <v>452.52553716383005</v>
+        <v>505.96762793760377</v>
       </c>
       <c r="D6" s="0">
-        <v>358908.32244935515</v>
+        <v>405615.17874309333</v>
       </c>
     </row>
     <row r="7">
@@ -548,13 +548,13 @@
         <v>25</v>
       </c>
       <c r="B7" s="0">
-        <v>812.51719945469085</v>
+        <v>821.13786384934338</v>
       </c>
       <c r="C7" s="0">
-        <v>504.93607747696512</v>
+        <v>558.66018993291607</v>
       </c>
       <c r="D7" s="0">
-        <v>410269.24757522048</v>
+        <v>458737.03497918317</v>
       </c>
     </row>
     <row r="8">
@@ -562,13 +562,13 @@
         <v>30</v>
       </c>
       <c r="B8" s="0">
-        <v>834.79379463241367</v>
+        <v>843.54367849010441</v>
       </c>
       <c r="C8" s="0">
-        <v>553.88007288036909</v>
+        <v>607.79742115900399</v>
       </c>
       <c r="D8" s="0">
-        <v>462375.64781108115</v>
+        <v>512703.67242126545</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         <v>35</v>
       </c>
       <c r="B9" s="0">
-        <v>859.76312529369409</v>
+        <v>868.67655374977267</v>
       </c>
       <c r="C9" s="0">
-        <v>599.13373360342587</v>
+        <v>653.19979673870864</v>
       </c>
       <c r="D9" s="0">
-        <v>515113.09127176099</v>
+        <v>567419.34834103345</v>
       </c>
     </row>
     <row r="10">
@@ -590,13 +590,13 @@
         <v>40</v>
       </c>
       <c r="B10" s="0">
-        <v>887.22578825402184</v>
+        <v>896.33045373357709</v>
       </c>
       <c r="C10" s="0">
-        <v>640.40136484783454</v>
+        <v>694.59474963182731</v>
       </c>
       <c r="D10" s="0">
-        <v>568180.6057260714</v>
+        <v>622586.42709845619</v>
       </c>
     </row>
     <row r="11">
@@ -604,13 +604,13 @@
         <v>45</v>
       </c>
       <c r="B11" s="0">
-        <v>916.96893076443519</v>
+        <v>926.28964065351954</v>
       </c>
       <c r="C11" s="0">
-        <v>677.35870942295389</v>
+        <v>731.67181597156514</v>
       </c>
       <c r="D11" s="0">
-        <v>621116.89152354375</v>
+        <v>677740.02349260915</v>
       </c>
     </row>
     <row r="12">
@@ -618,13 +618,13 @@
         <v>50</v>
       </c>
       <c r="B12" s="0">
-        <v>948.76532462207956</v>
+        <v>958.32628175210903</v>
       </c>
       <c r="C12" s="0">
-        <v>709.67373718544059</v>
+        <v>764.10845325444063</v>
       </c>
       <c r="D12" s="0">
-        <v>673313.83363650891</v>
+        <v>732265.21286268334</v>
       </c>
     </row>
     <row r="13">
@@ -632,13 +632,13 @@
         <v>55</v>
       </c>
       <c r="B13" s="0">
-        <v>982.37362214554162</v>
+        <v>992.20005358601952</v>
       </c>
       <c r="C13" s="0">
-        <v>737.01679849846698</v>
+        <v>791.58266390518656</v>
       </c>
       <c r="D13" s="0">
-        <v>724025.86192304979</v>
+        <v>785408.36154449021</v>
       </c>
     </row>
     <row r="14">
@@ -646,13 +646,13 @@
         <v>60</v>
       </c>
       <c r="B14" s="0">
-        <v>1017.5391703716315</v>
+        <v>1027.6587164183325</v>
       </c>
       <c r="C14" s="0">
-        <v>759.06479435716562</v>
+        <v>813.77860352897449</v>
       </c>
       <c r="D14" s="0">
-        <v>772378.16110850335</v>
+        <v>836286.67515128898</v>
       </c>
     </row>
     <row r="15">
@@ -660,13 +660,13 @@
         <v>65</v>
       </c>
       <c r="B15" s="0">
-        <v>1053.9950424142089</v>
+        <v>1064.4391626312222</v>
       </c>
       <c r="C15" s="0">
-        <v>775.50111635450025</v>
+        <v>830.38757818785336</v>
       </c>
       <c r="D15" s="0">
-        <v>817374.33202432783</v>
+        <v>883897.05838564713</v>
       </c>
     </row>
     <row r="16">
@@ -674,13 +674,13 @@
         <v>70</v>
       </c>
       <c r="B16" s="0">
-        <v>1091.4630303772233</v>
+        <v>1102.2686409145833</v>
       </c>
       <c r="C16" s="0">
-        <v>786.01167976574811</v>
+        <v>841.10510406984304</v>
       </c>
       <c r="D16" s="0">
-        <v>857902.68990901508</v>
+        <v>927123.77992938506</v>
       </c>
     </row>
     <row r="17">
@@ -688,13 +688,13 @@
         <v>75</v>
       </c>
       <c r="B17" s="0">
-        <v>1129.6543193869115</v>
+        <v>1140.8659045817494</v>
       </c>
       <c r="C17" s="0">
-        <v>793.79861087035783</v>
+        <v>845.62363006229771</v>
       </c>
       <c r="D17" s="0">
-        <v>896718.02949302993</v>
+        <v>964743.16764672589</v>
       </c>
     </row>
     <row r="18">
@@ -702,13 +702,13 @@
         <v>80</v>
       </c>
       <c r="B18" s="0">
-        <v>1168.2694286799262</v>
+        <v>1179.941973414323</v>
       </c>
       <c r="C18" s="0">
-        <v>796.83450709137242</v>
+        <v>843.61949431043649</v>
       </c>
       <c r="D18" s="0">
-        <v>930917.39435208833</v>
+        <v>995422.05092744972</v>
       </c>
     </row>
     <row r="19">
@@ -716,13 +716,13 @@
         <v>85</v>
       </c>
       <c r="B19" s="0">
-        <v>1206.9966952336056</v>
+        <v>1219.2000060937144</v>
       </c>
       <c r="C19" s="0">
-        <v>793.67001186378479</v>
+        <v>834.73123010602205</v>
       </c>
       <c r="D19" s="0">
-        <v>957957.08142560476</v>
+        <v>1017704.3208318758</v>
       </c>
     </row>
     <row r="20">
@@ -730,13 +730,13 @@
         <v>90</v>
       </c>
       <c r="B20" s="0">
-        <v>1245.5078988954351</v>
+        <v>1258.3333360390548</v>
       </c>
       <c r="C20" s="0">
-        <v>784.04360861304622</v>
+        <v>818.52377466435041</v>
       </c>
       <c r="D20" s="0">
-        <v>976532.50760603009</v>
+        <v>1029975.7520006716</v>
       </c>
     </row>
     <row r="21">
@@ -744,13 +744,13 @@
         <v>95</v>
       </c>
       <c r="B21" s="0">
-        <v>1307.1893226825234</v>
+        <v>1320.7609342425303</v>
       </c>
       <c r="C21" s="0">
-        <v>767.62883396882</v>
+        <v>794.42806420496663</v>
       </c>
       <c r="D21" s="0">
-        <v>1003436.215547277</v>
+        <v>1049249.5522678366</v>
       </c>
     </row>
     <row r="22">
@@ -758,13 +758,13 @@
         <v>100</v>
       </c>
       <c r="B22" s="0">
-        <v>1367.7147950669782</v>
+        <v>1382.2090872802974</v>
       </c>
       <c r="C22" s="0">
-        <v>743.96612021033957</v>
+        <v>761.63452648959378</v>
       </c>
       <c r="D22" s="0">
-        <v>1017533.4696402595</v>
+        <v>1052738.1637003429</v>
       </c>
     </row>
     <row r="23">
@@ -772,13 +772,13 @@
         <v>105</v>
       </c>
       <c r="B23" s="0">
-        <v>1426.3997848583081</v>
+        <v>1442.0841267439018</v>
       </c>
       <c r="C23" s="0">
-        <v>712.33102031441308</v>
+        <v>718.89286450308293</v>
       </c>
       <c r="D23" s="0">
-        <v>1016068.8141243779</v>
+        <v>1036703.9887293505</v>
       </c>
     </row>
     <row r="24">
@@ -786,13 +786,13 @@
         <v>110</v>
       </c>
       <c r="B24" s="0">
-        <v>1482.3338326520243</v>
+        <v>1499.6506324499846</v>
       </c>
       <c r="C24" s="0">
-        <v>671.45323989271492</v>
+        <v>664.10046455938846</v>
       </c>
       <c r="D24" s="0">
-        <v>995317.85453678714</v>
+        <v>995918.68168681546</v>
       </c>
     </row>
     <row r="25">
@@ -800,13 +800,13 @@
         <v>115</v>
       </c>
       <c r="B25" s="0">
-        <v>1534.0190566554104</v>
+        <v>1553.8054085868216</v>
       </c>
       <c r="C25" s="0">
-        <v>618.82450138813113</v>
+        <v>611.42682983656334</v>
       </c>
       <c r="D25" s="0">
-        <v>949288.57785467559</v>
+        <v>950038.31515514641</v>
       </c>
     </row>
     <row r="26">
@@ -814,13 +814,13 @@
         <v>120</v>
       </c>
       <c r="B26" s="0">
-        <v>1578.0613435288069</v>
+        <v>1602.3103506098066</v>
       </c>
       <c r="C26" s="0">
-        <v>548.54007705640459</v>
+        <v>546.13608401825934</v>
       </c>
       <c r="D26" s="0">
-        <v>865629.89097902505</v>
+        <v>875079.50026396394</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Question 7. Output is reverse calculated from the location of pin A in the original link, instead of being a convergence across 3 DOF's. We're goated
</commit_message>
<xml_diff>
--- a/Interim3/ENME473_Q7_BoxDimensions.xlsx
+++ b/Interim3/ENME473_Q7_BoxDimensions.xlsx
@@ -478,13 +478,13 @@
         <v>0</v>
       </c>
       <c r="B2" s="0">
-        <v>761.23831235875093</v>
+        <v>832.46895056959727</v>
       </c>
       <c r="C2" s="0">
-        <v>227.85929594485208</v>
+        <v>137.11917205240047</v>
       </c>
       <c r="D2" s="0">
-        <v>173455.22590031236</v>
+        <v>114147.45326143387</v>
       </c>
     </row>
     <row r="3">
@@ -492,13 +492,13 @@
         <v>5</v>
       </c>
       <c r="B3" s="0">
-        <v>763.55377057003204</v>
+        <v>836.24929120518345</v>
       </c>
       <c r="C3" s="0">
-        <v>321.59868152706906</v>
+        <v>240.78935819092459</v>
       </c>
       <c r="D3" s="0">
-        <v>245557.88589034448</v>
+        <v>201359.93011691171</v>
       </c>
     </row>
     <row r="4">
@@ -506,13 +506,13 @@
         <v>10</v>
       </c>
       <c r="B4" s="0">
-        <v>772.44581823758108</v>
+        <v>845.49858312141623</v>
       </c>
       <c r="C4" s="0">
-        <v>389.13234938420442</v>
+        <v>309.75261914314609</v>
       </c>
       <c r="D4" s="0">
-        <v>300583.65602279408</v>
+        <v>261895.4006036777</v>
       </c>
     </row>
     <row r="5">
@@ -520,13 +520,13 @@
         <v>15</v>
       </c>
       <c r="B5" s="0">
-        <v>785.33569826039775</v>
+        <v>858.4401461782328</v>
       </c>
       <c r="C5" s="0">
-        <v>449.67442900751735</v>
+        <v>370.74467979663336</v>
       </c>
       <c r="D5" s="0">
-        <v>353145.38169446431</v>
+        <v>318262.11711942405</v>
       </c>
     </row>
     <row r="6">
@@ -534,13 +534,13 @@
         <v>20</v>
       </c>
       <c r="B6" s="0">
-        <v>801.66231265908982</v>
+        <v>874.67903719724472</v>
       </c>
       <c r="C6" s="0">
-        <v>505.96762793760377</v>
+        <v>427.15835056453733</v>
       </c>
       <c r="D6" s="0">
-        <v>405615.17874309333</v>
+        <v>373626.45480255265</v>
       </c>
     </row>
     <row r="7">
@@ -548,13 +548,13 @@
         <v>25</v>
       </c>
       <c r="B7" s="0">
-        <v>821.13786384934338</v>
+        <v>893.98616237047918</v>
       </c>
       <c r="C7" s="0">
-        <v>558.66018993291607</v>
+        <v>479.8175876563248</v>
       </c>
       <c r="D7" s="0">
-        <v>458737.03497918317</v>
+        <v>428950.28382673883</v>
       </c>
     </row>
     <row r="8">
@@ -562,13 +562,13 @@
         <v>30</v>
       </c>
       <c r="B8" s="0">
-        <v>843.54367849010441</v>
+        <v>916.16847861785027</v>
       </c>
       <c r="C8" s="0">
-        <v>607.79742115900399</v>
+        <v>528.8351082637148</v>
       </c>
       <c r="D8" s="0">
-        <v>512703.67242126545</v>
+        <v>484502.05657767371</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         <v>35</v>
       </c>
       <c r="B9" s="0">
-        <v>868.67655374977267</v>
+        <v>941.03491745786221</v>
       </c>
       <c r="C9" s="0">
-        <v>653.19979673870864</v>
+        <v>574.06214941368796</v>
       </c>
       <c r="D9" s="0">
-        <v>567419.34834103345</v>
+        <v>540212.52738919284</v>
       </c>
     </row>
     <row r="10">
@@ -590,13 +590,13 @@
         <v>40</v>
       </c>
       <c r="B10" s="0">
-        <v>896.33045373357709</v>
+        <v>968.38498361179211</v>
       </c>
       <c r="C10" s="0">
-        <v>694.59474963182731</v>
+        <v>615.24156528877461</v>
       </c>
       <c r="D10" s="0">
-        <v>622586.42709845619</v>
+        <v>595790.69311946328</v>
       </c>
     </row>
     <row r="11">
@@ -604,13 +604,13 @@
         <v>45</v>
       </c>
       <c r="B11" s="0">
-        <v>926.28964065351954</v>
+        <v>998.00473693582944</v>
       </c>
       <c r="C11" s="0">
-        <v>731.67181597156514</v>
+        <v>652.07090510774265</v>
       </c>
       <c r="D11" s="0">
-        <v>677740.02349260915</v>
+        <v>650769.85211556091</v>
       </c>
     </row>
     <row r="12">
@@ -618,13 +618,13 @@
         <v>50</v>
       </c>
       <c r="B12" s="0">
-        <v>958.32628175210903</v>
+        <v>1029.665668583041</v>
       </c>
       <c r="C12" s="0">
-        <v>764.10845325444063</v>
+        <v>684.23163816716215</v>
       </c>
       <c r="D12" s="0">
-        <v>732265.21286268334</v>
+        <v>704529.82717906043</v>
       </c>
     </row>
     <row r="13">
@@ -632,13 +632,13 @@
         <v>55</v>
       </c>
       <c r="B13" s="0">
-        <v>992.20005358601952</v>
+        <v>1063.1248515370469</v>
       </c>
       <c r="C13" s="0">
-        <v>791.58266390518656</v>
+        <v>711.40338890365251</v>
       </c>
       <c r="D13" s="0">
-        <v>785408.36154449021</v>
+        <v>756310.62221114757</v>
       </c>
     </row>
     <row r="14">
@@ -646,13 +646,13 @@
         <v>60</v>
       </c>
       <c r="B14" s="0">
-        <v>1027.6587164183325</v>
+        <v>1098.1256709271816</v>
       </c>
       <c r="C14" s="0">
-        <v>813.77860352897449</v>
+        <v>733.27035737934352</v>
       </c>
       <c r="D14" s="0">
-        <v>836286.67515128898</v>
+        <v>805223.00316820585</v>
       </c>
     </row>
     <row r="15">
@@ -660,13 +660,13 @@
         <v>65</v>
       </c>
       <c r="B15" s="0">
-        <v>1064.4391626312222</v>
+        <v>1134.3987664542697</v>
       </c>
       <c r="C15" s="0">
-        <v>830.38757818785336</v>
+        <v>750.82377471453344</v>
       </c>
       <c r="D15" s="0">
-        <v>883897.05838564713</v>
+        <v>851733.56386070524</v>
       </c>
     </row>
     <row r="16">
@@ -674,13 +674,13 @@
         <v>70</v>
       </c>
       <c r="B16" s="0">
-        <v>1102.2686409145833</v>
+        <v>1171.6629202825986</v>
       </c>
       <c r="C16" s="0">
-        <v>841.10510406984304</v>
+        <v>765.73376426729487</v>
       </c>
       <c r="D16" s="0">
-        <v>927123.77992938506</v>
+        <v>897181.85840040573</v>
       </c>
     </row>
     <row r="17">
@@ -688,13 +688,13 @@
         <v>75</v>
       </c>
       <c r="B17" s="0">
-        <v>1140.8659045817494</v>
+        <v>1209.625607514449</v>
       </c>
       <c r="C17" s="0">
-        <v>845.62363006229771</v>
+        <v>774.94579514457632</v>
       </c>
       <c r="D17" s="0">
-        <v>964743.16764672589</v>
+        <v>937394.27824252588</v>
       </c>
     </row>
     <row r="18">
@@ -702,13 +702,13 @@
         <v>80</v>
       </c>
       <c r="B18" s="0">
-        <v>1179.941973414323</v>
+        <v>1247.9828049298872</v>
       </c>
       <c r="C18" s="0">
-        <v>843.61949431043649</v>
+        <v>778.24507525756667</v>
       </c>
       <c r="D18" s="0">
-        <v>995422.05092744972</v>
+        <v>971236.47194280918</v>
       </c>
     </row>
     <row r="19">
@@ -716,13 +716,13 @@
         <v>85</v>
       </c>
       <c r="B19" s="0">
-        <v>1219.2000060937144</v>
+        <v>1286.4173727909151</v>
       </c>
       <c r="C19" s="0">
-        <v>834.73123010602205</v>
+        <v>775.41778683455345</v>
       </c>
       <c r="D19" s="0">
-        <v>1017704.3208318758</v>
+        <v>997510.91215505206</v>
       </c>
     </row>
     <row r="20">
@@ -730,13 +730,13 @@
         <v>90</v>
       </c>
       <c r="B20" s="0">
-        <v>1258.3333360390548</v>
+        <v>1324.5947280552086</v>
       </c>
       <c r="C20" s="0">
-        <v>818.52377466435041</v>
+        <v>766.23335667400693</v>
       </c>
       <c r="D20" s="0">
-        <v>1029975.7520006716</v>
+        <v>1014948.6647104359</v>
       </c>
     </row>
     <row r="21">
@@ -744,13 +744,13 @@
         <v>95</v>
       </c>
       <c r="B21" s="0">
-        <v>1320.7609342425303</v>
+        <v>1385.8944483759385</v>
       </c>
       <c r="C21" s="0">
-        <v>794.42806420496663</v>
+        <v>750.41426091137441</v>
       </c>
       <c r="D21" s="0">
-        <v>1049249.5522678366</v>
+        <v>1039994.9581792068</v>
       </c>
     </row>
     <row r="22">
@@ -758,13 +758,13 @@
         <v>100</v>
       </c>
       <c r="B22" s="0">
-        <v>1382.2090872802974</v>
+        <v>1445.9853774056996</v>
       </c>
       <c r="C22" s="0">
-        <v>761.63452648959378</v>
+        <v>727.58272619971535</v>
       </c>
       <c r="D22" s="0">
-        <v>1052738.1637003429</v>
+        <v>1052073.9829377632</v>
       </c>
     </row>
     <row r="23">
@@ -772,13 +772,13 @@
         <v>105</v>
       </c>
       <c r="B23" s="0">
-        <v>1442.0841267439018</v>
+        <v>1504.1865450010093</v>
       </c>
       <c r="C23" s="0">
-        <v>718.89286450308293</v>
+        <v>697.16094635783361</v>
       </c>
       <c r="D23" s="0">
-        <v>1036703.9887293505</v>
+        <v>1048660.1152116237</v>
       </c>
     </row>
     <row r="24">
@@ -786,13 +786,13 @@
         <v>110</v>
       </c>
       <c r="B24" s="0">
-        <v>1499.6506324499846</v>
+        <v>1559.6227044165041</v>
       </c>
       <c r="C24" s="0">
-        <v>664.10046455938846</v>
+        <v>658.16769180109384</v>
       </c>
       <c r="D24" s="0">
-        <v>995918.68168681546</v>
+        <v>1026493.2754463902</v>
       </c>
     </row>
     <row r="25">
@@ -800,13 +800,13 @@
         <v>115</v>
       </c>
       <c r="B25" s="0">
-        <v>1553.8054085868216</v>
+        <v>1610.9512582816076</v>
       </c>
       <c r="C25" s="0">
-        <v>611.42682983656334</v>
+        <v>608.74958206735619</v>
       </c>
       <c r="D25" s="0">
-        <v>950038.31515514641</v>
+        <v>980665.90520981024</v>
       </c>
     </row>
     <row r="26">
@@ -814,13 +814,13 @@
         <v>120</v>
       </c>
       <c r="B26" s="0">
-        <v>1602.3103506098066</v>
+        <v>1655.4905653908636</v>
       </c>
       <c r="C26" s="0">
-        <v>546.13608401825934</v>
+        <v>544.87455903441446</v>
       </c>
       <c r="D26" s="0">
-        <v>875079.50026396394</v>
+        <v>902034.69180298026</v>
       </c>
     </row>
   </sheetData>

</xml_diff>